<commit_message>
docs: complete exception list E16-E18 in business-rules
</commit_message>
<xml_diff>
--- a/examples/demo/output/进销存台账.xlsx
+++ b/examples/demo/output/进销存台账.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3045c0121abc</t>
+          <t>4c648e2dabdd</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:03</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
     </row>
@@ -736,12 +736,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>B20261027172705</t>
+          <t>B20261027172854</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:55</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:55</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:55</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:55</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:55</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:07</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:07</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:07</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:07</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:07</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:03</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1742,12 +1742,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认期初; 批次: B20261027172704-000001</t>
+          <t>用户确认: 用户确认期初; 批次: B20261027172853-000001</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>B20261027172704-000001</t>
+          <t>B20261027172853-000001</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1821,12 +1821,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027172704-000002</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027172853-000002</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>B20261027172704-000002</t>
+          <t>B20261027172853-000002</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1900,12 +1900,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027172704-000003</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027172854-000003</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>B20261027172704-000003</t>
+          <t>B20261027172854-000003</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>批次:B20261027172705</t>
+          <t>批次:B20261027172854</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1984,12 +1984,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027172705-000004</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027172854-000004</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>B20261027172705-000004</t>
+          <t>B20261027172854-000004</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>批次:B20261027172705</t>
+          <t>批次:B20261027172854</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2068,12 +2068,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027172705-000005</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027172854-000005</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>B20261027172705-000005</t>
+          <t>B20261027172854-000005</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>批次:B20261027172705</t>
+          <t>批次:B20261027172854</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2152,12 +2152,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调拨; 批次: B20261027172705-000006</t>
+          <t>用户确认: 用户确认调拨; 批次: B20261027172854-000006</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>B20261027172705-000006</t>
+          <t>B20261027172854-000006</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>批次:B20261027172705</t>
+          <t>批次:B20261027172854</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2236,12 +2236,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调整; 批次: B20261027172705-000007</t>
+          <t>用户确认: 用户确认调整; 批次: B20261027172854-000007</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>B20261027172705-000007</t>
+          <t>B20261027172854-000007</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2315,12 +2315,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认费用; 批次: B20261027172705-000008</t>
+          <t>用户确认: 用户确认费用; 批次: B20261027172854-000008</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>B20261027172705-000008</t>
+          <t>B20261027172854-000008</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:55</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:55</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2473,12 +2473,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027172706-000009</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027172856-000009</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>B20261027172706-000009</t>
+          <t>B20261027172856-000009</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2520,7 +2520,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>批次:B20261027172706</t>
+          <t>批次:B20261027172856</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2557,12 +2557,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027172706-000010</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027172856-000010</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>B20261027172706-000010</t>
+          <t>B20261027172856-000010</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>B20261027172704-000001</t>
+          <t>B20261027172853-000001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B20261027172704-000002</t>
+          <t>B20261027172853-000002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B20261027172704-000003</t>
+          <t>B20261027172854-000003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2795,7 +2795,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B20261027172705-000004</t>
+          <t>B20261027172854-000004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B20261027172705-000005</t>
+          <t>B20261027172854-000005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B20261027172705-000006</t>
+          <t>B20261027172854-000006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B20261027172705-000007</t>
+          <t>B20261027172854-000007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B20261027172705-000008</t>
+          <t>B20261027172854-000008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B20261027172706-000009</t>
+          <t>B20261027172856-000009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B20261027172706-000010</t>
+          <t>B20261027172856-000010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:55</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:07</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:03</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
     </row>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
     </row>
@@ -3631,12 +3631,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>B20261027172704</t>
+          <t>B20261027172853</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -3702,12 +3702,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>B20261027172704</t>
+          <t>B20261027172853</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -3773,12 +3773,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>B20261027172704</t>
+          <t>B20261027172853</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -4018,12 +4018,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>B20261027172704</t>
+          <t>B20261027172853</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -4112,12 +4112,12 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>B20261027172704</t>
+          <t>B20261027172853</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:53</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -4206,12 +4206,12 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>B20261027172704</t>
+          <t>B20261027172854</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:04</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -4300,12 +4300,12 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>B20261027172706</t>
+          <t>B20261027172856</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -4561,12 +4561,12 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>B20261027172705</t>
+          <t>B20261027172854</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -4666,12 +4666,12 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>B20261027172705</t>
+          <t>B20261027172854</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -4771,12 +4771,12 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>B20261027172705</t>
+          <t>B20261027172854</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -4876,12 +4876,12 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>B20261027172706</t>
+          <t>B20261027172856</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:06</t>
+          <t>2026-10-27 17:28:56</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -5077,12 +5077,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>B20261027172705</t>
+          <t>B20261027172854</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -5293,12 +5293,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>B20261027172705</t>
+          <t>B20261027172854</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:27:05</t>
+          <t>2026-10-27 17:28:54</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">

</xml_diff>

<commit_message>
fix: persist audit rows for init/close/reopen (audit before save); docs: out_qty/out_cost口径; regression test
</commit_message>
<xml_diff>
--- a/examples/demo/output/进销存台账.xlsx
+++ b/examples/demo/output/进销存台账.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4c648e2dabdd</t>
+          <t>eed13d0a8e15</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:41</t>
         </is>
       </c>
     </row>
@@ -736,12 +736,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>B20261027172854</t>
+          <t>B20261027174443</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:55</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:55</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:55</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:55</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:55</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:45</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:45</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:45</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:45</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:45</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:41</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>sku</t>
+          <t>init</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1547,12 +1547,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>新增商品 SKU-001 (演示商品甲, 单位 件)</t>
+          <t>初始化台账 演示商贸有限公司 起始期间 2026-01</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>创建工作表与元数据</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>SKU-001</t>
+          <t>output/进销存台账.xlsx</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1569,7 +1574,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:41</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1584,12 +1589,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>新增商品 SKU-002 (演示商品乙, 单位 个)</t>
+          <t>新增商品 SKU-001 (演示商品甲, 单位 件)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>SKU-002</t>
+          <t>SKU-001</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1606,12 +1611,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:41</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>wh</t>
+          <t>sku</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1621,12 +1626,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>新增仓库 W01 (主仓)</t>
+          <t>新增商品 SKU-002 (演示商品乙, 单位 个)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>W01</t>
+          <t>SKU-002</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1643,7 +1648,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1658,12 +1663,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>新增仓库 W02 (分仓)</t>
+          <t>新增仓库 W01 (主仓)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>W02</t>
+          <t>W01</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1680,12 +1685,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>opening</t>
+          <t>wh</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1695,17 +1700,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>设置期初库存 2026-01 共 3 条</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>用户确认: 用户确认期初</t>
+          <t>新增仓库 W02 (分仓)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>P2026-01</t>
+          <t>W02</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1722,12 +1722,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>opening</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1737,17 +1737,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>导入 opening 文件 01_期初.csv =&gt; 成功 3, 拒绝 0, 待确认 0</t>
+          <t>设置期初库存 2026-01 共 3 条</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认期初; 批次: B20261027172853-000001</t>
+          <t>用户确认: 用户确认期初</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>B20261027172853-000001</t>
+          <t>P2026-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>purchase</t>
+          <t>import</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1779,12 +1779,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>采购入库 2 条</t>
+          <t>导入 opening 文件 01_期初.csv =&gt; 成功 3, 拒绝 0, 待确认 0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 首单: IN-000001</t>
+          <t>用户确认: 用户确认期初; 批次: B20261027174442-000001</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>B20261027174442-000001</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1801,12 +1806,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>purchase</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1816,17 +1821,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>导入 purchase 文件 02_采购_01.csv =&gt; 成功 2, 拒绝 0, 待确认 0</t>
+          <t>采购入库 2 条</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027172853-000002</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>B20261027172853-000002</t>
+          <t>用户确认: 用户确认采购; 首单: IN-000001</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1843,12 +1843,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>purchase</t>
+          <t>import</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1858,12 +1858,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>采购入库 1 条</t>
+          <t>导入 purchase 文件 02_采购_01.csv =&gt; 成功 2, 拒绝 0, 待确认 0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 首单: IN-000003</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027174442-000002</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>B20261027174442-000002</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1880,12 +1885,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>purchase</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1895,17 +1900,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>导入 purchase 文件 03_采购_02.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
+          <t>采购入库 1 条</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027172854-000003</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>B20261027172854-000003</t>
+          <t>用户确认: 用户确认采购; 首单: IN-000003</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1922,12 +1922,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>sale</t>
+          <t>import</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1937,17 +1937,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>销售出库 2 条</t>
+          <t>导入 purchase 文件 03_采购_02.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027174442-000003</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>批次:B20261027172854</t>
+          <t>B20261027174442-000003</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1964,12 +1964,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>sale</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1979,17 +1979,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>导入 sale 文件 04_销售_01.csv =&gt; 成功 2, 拒绝 0, 待确认 0</t>
+          <t>销售出库 2 条</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027172854-000004</t>
+          <t>用户确认: 用户确认销售</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>B20261027172854-000004</t>
+          <t>批次:B20261027174442</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2006,12 +2006,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>sale</t>
+          <t>import</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2021,17 +2021,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>销售出库 1 条</t>
+          <t>导入 sale 文件 04_销售_01.csv =&gt; 成功 2, 拒绝 0, 待确认 0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027174442-000004</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>批次:B20261027172854</t>
+          <t>B20261027174442-000004</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2048,12 +2048,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>sale</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2063,17 +2063,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>导入 sale 文件 05_销售_02.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
+          <t>销售出库 1 条</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027172854-000005</t>
+          <t>用户确认: 用户确认销售</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>B20261027172854-000005</t>
+          <t>批次:B20261027174443</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2090,12 +2090,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>transfer</t>
+          <t>import</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2105,17 +2105,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>仓库调拨 1 条(双边原子写入)</t>
+          <t>导入 sale 文件 05_销售_02.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调拨</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027174443-000005</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>批次:B20261027172854</t>
+          <t>B20261027174443-000005</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2132,12 +2132,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>transfer</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2147,17 +2147,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>导入 transfer 文件 06_调拨.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
+          <t>仓库调拨 1 条(双边原子写入)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调拨; 批次: B20261027172854-000006</t>
+          <t>用户确认: 用户确认调拨</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>B20261027172854-000006</t>
+          <t>批次:B20261027174443</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>adjust</t>
+          <t>import</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2189,17 +2189,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>库存调整 1 条</t>
+          <t>导入 transfer 文件 06_调拨.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调整</t>
+          <t>用户确认: 用户确认调拨; 批次: B20261027174443-000006</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>批次:B20261027172854</t>
+          <t>B20261027174443-000006</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2216,12 +2216,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>adjust</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2231,17 +2231,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>导入 adjust 文件 07_调整.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
+          <t>库存调整 1 条</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调整; 批次: B20261027172854-000007</t>
+          <t>用户确认: 用户确认调整</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>B20261027172854-000007</t>
+          <t>批次:B20261027174443</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2258,12 +2258,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>fee</t>
+          <t>import</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2273,12 +2273,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>登记附加费用 1 张(待分摊)</t>
+          <t>导入 adjust 文件 07_调整.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认费用</t>
+          <t>用户确认: 用户确认调整; 批次: B20261027174443-000007</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>B20261027174443-000007</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2295,12 +2300,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>fee</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2310,17 +2315,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>导入 fee 文件 08_费用.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
+          <t>登记附加费用 1 张(待分摊)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认费用; 批次: B20261027172854-000008</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>B20261027172854-000008</t>
+          <t>用户确认: 用户确认费用</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2337,12 +2337,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:55</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>fee_alloc</t>
+          <t>import</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2352,17 +2352,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>附加费用分摊 FEE-000001 -&gt; PO-001 共 2 行, 规则 按数量比例, 总额 150.00</t>
+          <t>导入 fee 文件 08_费用.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认分摊; 明细: {'IN-000001': Decimal('75.00'), 'IN-000002': Decimal('75.00')}</t>
+          <t>用户确认: 用户确认费用; 批次: B20261027174443-000008</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>FEE-000001</t>
+          <t>B20261027174443-000008</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2379,12 +2379,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:55</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>period</t>
+          <t>fee_alloc</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2394,12 +2394,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>开启期间 2026-02</t>
+          <t>附加费用分摊 FEE-000001 -&gt; PO-001 共 2 行, 规则 按数量比例, 总额 150.00</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>用户确认: 用户确认分摊; 明细: {'IN-000001': Decimal('75.00'), 'IN-000002': Decimal('75.00')}</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>FEE-000001</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2416,12 +2421,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>purchase</t>
+          <t>close</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2431,12 +2436,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>采购入库 1 条</t>
+          <t>正式结账 2026-01 (版本 1)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 首单: IN-000004</t>
+          <t>用户确认: 用户确认结账; 写回出库成本与月末结存</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>P2026-01</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2453,12 +2463,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>import</t>
+          <t>period</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2468,17 +2478,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>导入 purchase 文件 09_下月采购.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027172856-000009</t>
+          <t>开启期间 2026-02</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>B20261027172856-000009</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2495,12 +2500,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>sale</t>
+          <t>purchase</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2510,17 +2515,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>销售出库 1 条</t>
+          <t>采购入库 1 条</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>批次:B20261027172856</t>
+          <t>用户确认: 用户确认采购; 首单: IN-000004</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2552,20 +2552,146 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>导入 purchase 文件 09_下月采购.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>用户确认: 用户确认采购; 批次: B20261027174444-000009</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>B20261027174444-000009</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>OP-000027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:44:44</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>销售出库 1 条</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>用户确认: 用户确认销售</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>批次:B20261027174444</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>OP-000028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:44:44</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>import</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
           <t>导入 sale 文件 10_下月销售.csv =&gt; 成功 1, 拒绝 0, 待确认 0</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027172856-000010</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>B20261027172856-000010</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>用户确认: 用户确认销售; 批次: B20261027174444-000010</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>B20261027174444-000010</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>OP-000029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:44:45</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>close</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>正式结账 2026-02 (版本 1)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>用户确认: 用户确认结账; 写回出库成本与月末结存</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>P2026-02</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
         <is>
           <t>成功</t>
         </is>
@@ -2655,7 +2781,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>B20261027172853-000001</t>
+          <t>B20261027174442-000001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2687,7 +2813,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -2709,7 +2835,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B20261027172853-000002</t>
+          <t>B20261027174442-000002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2741,7 +2867,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -2763,7 +2889,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B20261027172854-000003</t>
+          <t>B20261027174442-000003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2795,7 +2921,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -2817,7 +2943,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B20261027172854-000004</t>
+          <t>B20261027174442-000004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2849,7 +2975,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -2871,7 +2997,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B20261027172854-000005</t>
+          <t>B20261027174443-000005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2903,7 +3029,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -2925,7 +3051,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B20261027172854-000006</t>
+          <t>B20261027174443-000006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2957,7 +3083,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -2979,7 +3105,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B20261027172854-000007</t>
+          <t>B20261027174443-000007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3011,7 +3137,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -3033,7 +3159,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B20261027172854-000008</t>
+          <t>B20261027174443-000008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3065,7 +3191,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -3087,7 +3213,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B20261027172856-000009</t>
+          <t>B20261027174444-000009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3119,7 +3245,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -3141,7 +3267,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B20261027172856-000010</t>
+          <t>B20261027174444-000010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3173,7 +3299,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -3249,7 +3375,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:55</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3279,7 +3405,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:45</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -3362,7 +3488,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:41</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3515,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:41</t>
         </is>
       </c>
     </row>
@@ -3452,7 +3578,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3600,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
     </row>
@@ -3631,12 +3757,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>B20261027172853</t>
+          <t>B20261027174442</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -3702,12 +3828,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>B20261027172853</t>
+          <t>B20261027174442</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -3773,12 +3899,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>B20261027172853</t>
+          <t>B20261027174442</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -4018,12 +4144,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>B20261027172853</t>
+          <t>B20261027174442</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -4112,12 +4238,12 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>B20261027172853</t>
+          <t>B20261027174442</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:53</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -4206,12 +4332,12 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>B20261027172854</t>
+          <t>B20261027174442</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -4300,12 +4426,12 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>B20261027172856</t>
+          <t>B20261027174444</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -4561,12 +4687,12 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>B20261027172854</t>
+          <t>B20261027174442</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -4666,12 +4792,12 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>B20261027172854</t>
+          <t>B20261027174442</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:42</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -4771,12 +4897,12 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>B20261027172854</t>
+          <t>B20261027174443</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -4876,12 +5002,12 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>B20261027172856</t>
+          <t>B20261027174444</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:56</t>
+          <t>2026-10-27 17:44:44</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -5077,12 +5203,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>B20261027172854</t>
+          <t>B20261027174443</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -5293,12 +5419,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>B20261027172854</t>
+          <t>B20261027174443</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:28:54</t>
+          <t>2026-10-27 17:44:43</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">

</xml_diff>